<commit_message>
Atualiza instrução de trabalho
</commit_message>
<xml_diff>
--- a/Base/Backlog_14.xlsx
+++ b/Base/Backlog_14.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\franciscoj\Python_Initial\Pyhton_Web\Base\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0738208C-22C4-4ADE-A7C4-8FEE849CFCBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7627DB6A-7891-490A-9169-6294C36233B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="418" xr2:uid="{89A3EF9E-2AF9-420D-85DF-9BB5B68F651F}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="418" xr2:uid="{89A3EF9E-2AF9-420D-85DF-9BB5B68F651F}"/>
   </bookViews>
   <sheets>
     <sheet name="ITI" sheetId="2" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="25">
   <si>
     <t>Backlog</t>
   </si>
@@ -95,9 +95,6 @@
   </si>
   <si>
     <t>Jorgenaldo Reis</t>
-  </si>
-  <si>
-    <t>Erick Silva</t>
   </si>
   <si>
     <t>Felipe Nascimento</t>
@@ -606,7 +603,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C2" s="10">
         <v>2025</v>
@@ -630,7 +627,7 @@
         <v>45754</v>
       </c>
       <c r="J2" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K2" s="10" t="s">
         <v>11</v>
@@ -641,7 +638,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C3" s="10">
         <v>2025</v>
@@ -676,7 +673,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C4" s="10">
         <v>2025</v>
@@ -711,7 +708,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C5" s="10">
         <v>2025</v>
@@ -735,7 +732,7 @@
         <v>45754</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K5" s="10" t="s">
         <v>11</v>
@@ -746,7 +743,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C6" s="10">
         <v>2025</v>
@@ -770,7 +767,7 @@
         <v>45754</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K6" s="10" t="s">
         <v>11</v>
@@ -781,7 +778,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C7" s="10">
         <v>2025</v>
@@ -805,7 +802,7 @@
         <v>45754</v>
       </c>
       <c r="J7" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K7" s="10" t="s">
         <v>11</v>
@@ -816,7 +813,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C8" s="10">
         <v>2025</v>
@@ -840,7 +837,7 @@
         <v>45754</v>
       </c>
       <c r="J8" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K8" s="10" t="s">
         <v>11</v>
@@ -851,7 +848,7 @@
         <v>4</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C9" s="10">
         <v>2025</v>
@@ -875,7 +872,7 @@
         <v>45754</v>
       </c>
       <c r="J9" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K9" s="10" t="s">
         <v>11</v>
@@ -886,7 +883,7 @@
         <v>4</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C10" s="10">
         <v>2025</v>
@@ -910,7 +907,7 @@
         <v>45754</v>
       </c>
       <c r="J10" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K10" s="10" t="s">
         <v>11</v>
@@ -921,7 +918,7 @@
         <v>4</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C11" s="10">
         <v>2025</v>
@@ -956,7 +953,7 @@
         <v>4</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C12" s="10">
         <v>2025</v>
@@ -980,7 +977,7 @@
         <v>45754</v>
       </c>
       <c r="J12" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K12" s="10" t="s">
         <v>11</v>
@@ -991,7 +988,7 @@
         <v>4</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C13" s="10">
         <v>2025</v>
@@ -1026,7 +1023,7 @@
         <v>4</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C14" s="10">
         <v>2025</v>
@@ -1050,7 +1047,7 @@
         <v>45754</v>
       </c>
       <c r="J14" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K14" s="10" t="s">
         <v>11</v>
@@ -1061,7 +1058,7 @@
         <v>4</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C15" s="10">
         <v>2025</v>
@@ -1096,7 +1093,7 @@
         <v>4</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C16" s="10">
         <v>2025</v>
@@ -1120,7 +1117,7 @@
         <v>45754</v>
       </c>
       <c r="J16" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K16" s="10" t="s">
         <v>11</v>
@@ -1131,7 +1128,7 @@
         <v>4</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C17" s="10">
         <v>2025</v>
@@ -1155,7 +1152,7 @@
         <v>45754</v>
       </c>
       <c r="J17" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K17" s="10" t="s">
         <v>11</v>
@@ -1190,7 +1187,7 @@
         <v>45754</v>
       </c>
       <c r="J18" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K18" s="10" t="s">
         <v>11</v>
@@ -1236,7 +1233,7 @@
         <v>4</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C20" s="10">
         <v>2025</v>
@@ -1271,7 +1268,7 @@
         <v>4</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C21" s="10">
         <v>2025</v>
@@ -1295,7 +1292,7 @@
         <v>45754</v>
       </c>
       <c r="J21" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K21" s="10" t="s">
         <v>11</v>
@@ -1656,7 +1653,7 @@
         <v>14</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C2" s="10">
         <v>2025</v>
@@ -1680,7 +1677,7 @@
         <v>45754</v>
       </c>
       <c r="J2" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K2" s="10" t="s">
         <v>15</v>
@@ -1691,7 +1688,7 @@
         <v>14</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C3" s="10">
         <v>2025</v>
@@ -1715,7 +1712,7 @@
         <v>45754</v>
       </c>
       <c r="J3" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K3" s="10" t="s">
         <v>15</v>
@@ -1726,7 +1723,7 @@
         <v>14</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C4" s="10">
         <v>2025</v>
@@ -1750,7 +1747,7 @@
         <v>45754</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K4" s="10" t="s">
         <v>15</v>
@@ -1761,7 +1758,7 @@
         <v>14</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" s="10">
         <v>2025</v>
@@ -1785,7 +1782,7 @@
         <v>45754</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K5" s="10" t="s">
         <v>15</v>
@@ -1796,7 +1793,7 @@
         <v>14</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C6" s="10">
         <v>2025</v>

</xml_diff>